<commit_message>
backend Flask con Cloudinary integrado
</commit_message>
<xml_diff>
--- a/reportes.xlsx
+++ b/reportes.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,29 +479,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>99999997</t>
+          <t>8000000000</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2N99999</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>999999988</t>
-        </is>
-      </c>
+          <t>2N18001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>prueba de fotogrfias con rutas a aperturar desde el csv</t>
+          <t>prueba coudinary</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>13.7388045</v>
+        <v>13.740956</v>
       </c>
       <c r="F2" t="n">
-        <v>-89.1876425</v>
+        <v>-89.18454</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -509,7 +505,7 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>46132.16875056713</v>
+        <v>46173.22044858796</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -520,62 +516,66 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>97374398</t>
+          <t>900000000000</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2N14110</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>97603846</t>
-        </is>
-      </c>
+          <t>2N12111</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>No aparese en ruta es un servicio nuevo no eata en sistema lectura 0</t>
+          <t>Prueba de carga fotos</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>13.7046826</v>
+        <v>13.7377922</v>
       </c>
       <c r="F3" t="n">
-        <v>-88.5639304</v>
+        <v>-89.1892795</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2129CAESS</t>
+          <t>MORALESV00A</t>
         </is>
       </c>
       <c r="H3" s="1" t="n">
-        <v>46130.64524680556</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
+        <v>46172.93540412037</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>97502083</t>
+          <t>97594713</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2N13062</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>2n09069</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>95624058</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>No sé encuentra</t>
+          <t>3 meses y no aparese lectjfa 1</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>13.7287134</v>
+        <v>13.7174438</v>
       </c>
       <c r="F4" t="n">
-        <v>-88.9608185</v>
+        <v>-88.94312859999999</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -583,157 +583,1490 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>46129.74102649306</v>
+        <v>46155.61522716435</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>97375961</t>
+          <t>97594713</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2N13116</t>
+          <t>2n09069</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>97087622</t>
+          <t>95624058</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>No aparese en sistema lectura 205</t>
+          <t>3 meses y no aparese lectjfa 1</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>13.7763976</v>
+        <v>13.7174438</v>
       </c>
       <c r="F5" t="n">
-        <v>-88.5697462</v>
+        <v>-88.94312859999999</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2129CAESS</t>
+          <t>2125CAESS</t>
         </is>
       </c>
       <c r="H5" s="1" t="n">
-        <v>46129.60195969907</v>
+        <v>46155.61521583334</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>561</t>
+          <t>97084322</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2n11026</t>
+          <t>2N07064</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>561</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>95658515</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Lectura 630 asignarlo</t>
+        </is>
+      </c>
       <c r="E6" t="n">
-        <v>13.7152309</v>
+        <v>13.7314208</v>
       </c>
       <c r="F6" t="n">
-        <v>-89.2482759</v>
+        <v>-88.8869856</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2132CAESS</t>
+          <t>2125CAESS</t>
         </is>
       </c>
       <c r="H6" s="1" t="n">
-        <v>46127.82988920139</v>
+        <v>46153.75147538194</v>
       </c>
       <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>97006778</t>
+          <t>97606797</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2N0326</t>
+          <t>2N07086</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>95959595</t>
+          <t>95762787</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>No está en MRU</t>
+          <t>Asignar contiguo</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>13.7357458</v>
+        <v>13.9057587</v>
       </c>
       <c r="F7" t="n">
-        <v>-89.205091</v>
+        <v>-89.0351749</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2111CAESS</t>
+          <t>MORALESV00A</t>
         </is>
       </c>
       <c r="H7" s="1" t="n">
-        <v>46125.9176921875</v>
+        <v>46153.68422814815</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>612425</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2N01125</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>96113026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Lectura 1200</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>13.8757571</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-88.62473420000001</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>46142.72780292824</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>612425</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2N01125</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>96113026</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Lectura 1200</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>13.8757571</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-88.62473420000001</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>46142.72778704861</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>97612324</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2N21234</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>97654345</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Lectura 15</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>13.8757811</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-88.624723</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>46142.72772310185</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2134455</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nrin24447</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23473636</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>13.875793</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-88.6247224</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>46142.72760693287</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>97234336</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2N11124</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>96345432</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Lectura 102</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>13.8757512</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-88.6247303</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>46142.72760539352</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2134455</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Nrin24447</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>23473636</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>13.875793</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-88.6247224</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>46142.72760221065</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2134455</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nrin24447</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23473636</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>13.875793</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-88.6247224</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="n">
+        <v>46142.72759645833</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>97234336</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2N11124</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>96345432</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Lectura 102</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>13.8757512</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-88.6247303</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="n">
+        <v>46142.72757475694</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2134455</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Nrin24447</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>23473636</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>13.875793</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-88.6247224</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="n">
+        <v>46142.72756033565</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2134455</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Nrin24447</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>23473636</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>13.875793</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-88.6247224</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="n">
+        <v>46142.72755175926</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2134455</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Nrin24447</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>23473636</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>13.875793</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-88.6247224</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="n">
+        <v>46142.72754609954</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2134455</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Nrin24447</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23473636</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>13.875793</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-88.6247224</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>46142.72753142361</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>240130</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>N015077</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>120724</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medidor no está en ruta</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>13.7364911</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-89.0541063</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2126CAESS</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="n">
+        <v>46141.88838930555</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>25069000</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2n104038384</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>95091737</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Malo</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>13.7365609</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-89.05406290000001</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2126CAESS</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>46141.88713079861</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2N2030</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>96753612</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Medidor no aparece en ruta</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>13.7365175</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-89.0541212</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2126CAESS</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>46141.88704655092</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>25069000</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2N119080</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>563917638</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Medidor no me aparece en ruta</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>13.7365573038099</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-89.05407218858051</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>MORALESV00A</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="n">
+        <v>46141.88695648148</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>25069000</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2N119080</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>563917638</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Medidor no me aparece en ruta</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>13.7365573038099</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-89.05407218858051</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>MORALESV00A</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="n">
+        <v>46141.88692722222</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2125</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1314</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>13.7229729</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-88.9330645</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2125CAESS</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>46141.70855020834</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>José</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2125</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1314</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>13.7229729</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-88.9330645</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2125CAESS</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="n">
+        <v>46141.70852802083</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>799820</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2N16045</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>96992468</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Medidor se observa con bornera dañada, cliente dice q medidor echa chispas a veces, cambiar medidor.</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>14.0838638</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-88.91332269999999</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2124CAESS</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>46137.73896986111</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>799820</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2N16045</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>96992468</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Medidor se observa con bornera dañada, cliente dice q medidor echa chispas a veces, cambiar medidor.</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>14.0838638</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-88.91332269999999</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2124CAESS</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="n">
+        <v>46137.73891471065</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>95512318</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2N19020</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>687805</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No aparece en MRU</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>13.6950659</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-89.1490165</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2132CAESS</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>46136.81605353009</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>95512318</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2N19020</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>687805</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>No aparece en MRU</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>13.6950659</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-89.1490165</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2132CAESS</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>46136.81604326389</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>95512318</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2N19020</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>687805</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>No aparece en MRU</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>13.6950659</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-89.1490165</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2132CAESS</t>
+        </is>
+      </c>
+      <c r="H31" s="1" t="n">
+        <v>46136.8160140625</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>97376212</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2N17121</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>95948365</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>No aparese en la ruta lectura que tien el medidor es 273</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>13.8651126</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-88.6324272</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H32" s="1" t="n">
+        <v>46134.83288679398</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>97445328</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2N17073</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>96712022</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Lectura 10 servicio nuevo</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>13.7473387</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-89.106342</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>MORALESV00A</t>
+        </is>
+      </c>
+      <c r="H33" s="1" t="n">
+        <v>46134.71835181713</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>95595046</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2N20304</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>95354456</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Prueba</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>13.7358183</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-89.20502310000001</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>MORALESV00A</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="n">
+        <v>46132.56352863426</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>99999997</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2N99999</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>999999988</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>prueba de fotogrfias con rutas a aperturar desde el csv</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>13.7388045</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-89.1876425</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>MORALESV00A</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="n">
+        <v>46132.16875056713</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>ver foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>97374398</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2N14110</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>97603846</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>No aparese en ruta es un servicio nuevo no eata en sistema lectura 0</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>13.7046826</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-88.5639304</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="n">
+        <v>46130.64524680556</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>97502083</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2N13062</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>No sé encuentra</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>13.7287134</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-88.9608185</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2125CAESS</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="n">
+        <v>46129.74102649306</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>97375961</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2N13116</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>97087622</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>No aparese en sistema lectura 205</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>13.7763976</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-88.5697462</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2129CAESS</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="n">
+        <v>46129.60195969907</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>561</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2n11026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>561</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>13.7152309</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-89.2482759</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2132CAESS</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>46127.82988920139</v>
+      </c>
+      <c r="I39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>97006778</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2N0326</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>95959595</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>No está en MRU</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>13.7357458</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-89.205091</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2111CAESS</t>
+        </is>
+      </c>
+      <c r="H40" s="1" t="n">
+        <v>46125.9176921875</v>
+      </c>
+      <c r="I40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>99</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>2nprueba</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>98</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>No estaba en mru</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E41" t="n">
         <v>13.7357953</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F41" t="n">
         <v>-89.20505129999999</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>2111CAESS</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H41" s="1" t="n">
         <v>46125.91738023148</v>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>